<commit_message>
Update to ticket download and upload for 2026
</commit_message>
<xml_diff>
--- a/test/fixtures/files/invalid_tickets.xlsx
+++ b/test/fixtures/files/invalid_tickets.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
   <si>
     <t>Date</t>
   </si>
@@ -52,49 +52,52 @@
     <t>Booking Type</t>
   </si>
   <si>
+    <t>Question 15</t>
+  </si>
+  <si>
+    <t>Question 4</t>
+  </si>
+  <si>
+    <t>Question 1</t>
+  </si>
+  <si>
+    <t>Question 14</t>
+  </si>
+  <si>
+    <t>Question 13</t>
+  </si>
+  <si>
+    <t>Question 5</t>
+  </si>
+  <si>
+    <t>Question 6</t>
+  </si>
+  <si>
+    <t>Question 10</t>
+  </si>
+  <si>
     <t>Question 16</t>
   </si>
   <si>
-    <t>Question 6</t>
+    <t>Question 3</t>
+  </si>
+  <si>
+    <t>Question 7</t>
+  </si>
+  <si>
+    <t>Question 11</t>
+  </si>
+  <si>
+    <t>Question 9</t>
   </si>
   <si>
     <t>Question 8</t>
   </si>
   <si>
-    <t>Question 15</t>
-  </si>
-  <si>
-    <t>Question 14</t>
-  </si>
-  <si>
-    <t>Question 3</t>
-  </si>
-  <si>
-    <t>Question 9</t>
-  </si>
-  <si>
-    <t>Question 13</t>
-  </si>
-  <si>
     <t>Question 2</t>
   </si>
   <si>
-    <t>Question 7</t>
-  </si>
-  <si>
-    <t>Question 4</t>
-  </si>
-  <si>
     <t>Question 12</t>
-  </si>
-  <si>
-    <t>Question 10</t>
-  </si>
-  <si>
-    <t>Question 11</t>
-  </si>
-  <si>
-    <t>Question 1</t>
   </si>
   <si>
     <t>2/06/2023</t>
@@ -627,90 +630,90 @@
         <v>24</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H2" s="4">
         <v>417858583</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q2" s="4">
         <v>23</v>
       </c>
       <c r="R2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="S2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="W2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Y2" s="3"/>
       <c r="Z2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AB2" s="3"/>
     </row>

</xml_diff>